<commit_message>
Cleaned project: removed temp Excel file and added gitignore
</commit_message>
<xml_diff>
--- a/Excel_Analysis.xlsx
+++ b/Excel_Analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sakshi\Downloads\EXCEL project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sakshi\Downloads\ab-testing-landing-page-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4699CD4E-A988-4236-99E5-C51A400931B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6097FAA2-5B23-4A24-875F-4662A8638D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="original_ab_testing_dataset" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -123,7 +123,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -163,7 +163,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[original_ab_testing_dataset.xlsx]pivot!PivotTable1</c:name>
+    <c:name>[Excel_Analysis.xlsx]pivot!PivotTable1</c:name>
     <c:fmtId val="3"/>
   </c:pivotSource>
   <c:chart>
@@ -639,7 +639,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[original_ab_testing_dataset.xlsx]pivot!PivotTable2</c:name>
+    <c:name>[Excel_Analysis.xlsx]pivot!PivotTable2</c:name>
     <c:fmtId val="4"/>
   </c:pivotSource>
   <c:chart>
@@ -1111,7 +1111,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[original_ab_testing_dataset.xlsx]pivot!PivotTable3</c:name>
+    <c:name>[Excel_Analysis.xlsx]pivot!PivotTable3</c:name>
     <c:fmtId val="3"/>
   </c:pivotSource>
   <c:chart>
@@ -3415,13 +3415,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>144780</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>213360</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3448,16 +3448,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>274320</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>579120</xdr:colOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>525780</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3484,16 +3484,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>251460</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>205740</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -10902,6 +10902,64 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="E3:F6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of converted" fld="2" subtotal="average" baseField="1" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="4" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000002000000}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
@@ -10959,7 +11017,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="J3:K6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
@@ -10996,64 +11054,6 @@
   </dataFields>
   <chartFormats count="1">
     <chartFormat chart="3" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="E3:F6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="4">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of converted" fld="2" subtotal="average" baseField="1" baseItem="0" numFmtId="166"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="4" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">

</xml_diff>